<commit_message>
Track A churn sweep 2026-07-17
</commit_message>
<xml_diff>
--- a/data/FBS_SC_Database_v8_1_Clean.xlsx
+++ b/data/FBS_SC_Database_v8_1_Clean.xlsx
@@ -1683,69 +1683,73 @@
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="82" t="inlineStr">
         <is>
           <t>South Carolina</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="82" t="inlineStr">
         <is>
           <t>SEC</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr"/>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>Luke Day</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="C14" s="82" t="inlineStr"/>
+      <c r="D14" s="82" t="inlineStr">
+        <is>
+          <t>Jeff Dillman</t>
+        </is>
+      </c>
+      <c r="E14" s="82" t="inlineStr">
         <is>
           <t>Dir. of Athletic Performance</t>
         </is>
       </c>
-      <c r="F14" s="10" t="n">
+      <c r="F14" s="83" t="n">
         <v>450000</v>
       </c>
-      <c r="G14" s="9" t="n">
+      <c r="G14" s="82" t="n">
         <v>2024</v>
       </c>
-      <c r="H14" s="19" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="I14" s="9" t="inlineStr">
+      <c r="H14" s="84" t="inlineStr">
+        <is>
+          <t>Unverified</t>
+        </is>
+      </c>
+      <c r="I14" s="82" t="inlineStr">
         <is>
           <t>Mid ($350K-$499K)</t>
         </is>
       </c>
-      <c r="J14" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="K14" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="M14" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="N14" s="9" t="n">
+      <c r="J14" s="82" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="82" t="n">
+        <v>2</v>
+      </c>
+      <c r="M14" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="N14" s="82" t="n">
         <v>5</v>
       </c>
-      <c r="O14" s="12" t="inlineStr">
+      <c r="O14" s="88" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="P14" s="9" t="inlineStr">
+      <c r="P14" s="82" t="inlineStr">
         <is>
           <t>FootballScoop 2024. Shane Beamer still HC.</t>
         </is>
       </c>
-      <c r="Q14" s="9" t="inlineStr"/>
+      <c r="Q14" s="82" t="inlineStr">
+        <is>
+          <t>[Churn 2026-07-17] Name changed: Luke Day → Jeff Dillman. Salary cleared — requires verification.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="82" t="inlineStr">
@@ -2649,71 +2653,71 @@
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="A28" s="82" t="inlineStr">
         <is>
           <t>Penn State</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="82" t="inlineStr">
         <is>
           <t>Big Ten</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr"/>
-      <c r="D28" s="65" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="C28" s="82" t="inlineStr"/>
+      <c r="D28" s="85" t="inlineStr">
+        <is>
+          <t>Nittany Lions</t>
+        </is>
+      </c>
+      <c r="E28" s="82" t="inlineStr">
         <is>
           <t>Dir. of S&amp;C</t>
         </is>
       </c>
-      <c r="F28" s="66" t="n">
+      <c r="F28" s="89" t="n">
         <v>350000</v>
       </c>
-      <c r="G28" s="9" t="n">
+      <c r="G28" s="82" t="n">
         <v>2024</v>
       </c>
-      <c r="H28" s="11" t="inlineStr">
-        <is>
-          <t>Estimated</t>
-        </is>
-      </c>
-      <c r="I28" s="9" t="inlineStr">
+      <c r="H28" s="86" t="inlineStr">
+        <is>
+          <t>Unverified</t>
+        </is>
+      </c>
+      <c r="I28" s="82" t="inlineStr">
         <is>
           <t>Lower Power ($250K-$349K)</t>
         </is>
       </c>
-      <c r="J28" s="9" t="n">
+      <c r="J28" s="82" t="n">
         <v>3</v>
       </c>
-      <c r="K28" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="M28" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="N28" s="9" t="n">
+      <c r="K28" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="82" t="n">
+        <v>2</v>
+      </c>
+      <c r="M28" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="N28" s="82" t="n">
         <v>6</v>
       </c>
-      <c r="O28" s="12" t="inlineStr">
+      <c r="O28" s="88" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="P28" s="65" t="inlineStr">
+      <c r="P28" s="85" t="inlineStr">
         <is>
           <t>Franklin fired Oct 12 2025 (3-3 record). Chuck Losey followed Franklin to Virginia Tech. Penn State hired Matt Campbell from Iowa State (Dec 2025). Campbell likely brings new S&amp;C staff. Possibly Reid Kagy (ISU S&amp;C under Campbell) following to PSU — unconfirmed.</t>
         </is>
       </c>
-      <c r="Q28" s="65" t="inlineStr">
-        <is>
-          <t>Franklin fired Oct 2025; Losey to VT; Campbell new HC Dec 2025; new S&amp;C not confirmed.</t>
+      <c r="Q28" s="85" t="inlineStr">
+        <is>
+          <t>[Churn 2026-07-17] Name changed: Unknown → Nittany Lions. Salary cleared — requires verification.</t>
         </is>
       </c>
     </row>
@@ -3822,73 +3826,77 @@
       </c>
     </row>
     <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="14" t="inlineStr">
+      <c r="A45" s="82" t="inlineStr">
         <is>
           <t>Notre Dame</t>
         </is>
       </c>
-      <c r="B45" s="14" t="inlineStr">
+      <c r="B45" s="82" t="inlineStr">
         <is>
           <t>ACC</t>
         </is>
       </c>
-      <c r="C45" s="14" t="inlineStr">
+      <c r="C45" s="82" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D45" s="14" t="inlineStr">
-        <is>
-          <t>Sean Sutton</t>
-        </is>
-      </c>
-      <c r="E45" s="14" t="inlineStr">
+      <c r="D45" s="82" t="inlineStr">
+        <is>
+          <t>Before Notre Dame</t>
+        </is>
+      </c>
+      <c r="E45" s="82" t="inlineStr">
         <is>
           <t>Dir. of Athletic Performance</t>
         </is>
       </c>
-      <c r="F45" s="15" t="n">
+      <c r="F45" s="83" t="n">
         <v>550000</v>
       </c>
-      <c r="G45" s="14" t="n">
+      <c r="G45" s="82" t="n">
         <v>2024</v>
       </c>
-      <c r="H45" s="16" t="inlineStr">
+      <c r="H45" s="86" t="inlineStr">
+        <is>
+          <t>Unverified</t>
+        </is>
+      </c>
+      <c r="I45" s="82" t="inlineStr">
+        <is>
+          <t>Upper Mid ($500K-$699K)</t>
+        </is>
+      </c>
+      <c r="J45" s="82" t="n">
+        <v>4</v>
+      </c>
+      <c r="K45" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="L45" s="82" t="n">
+        <v>2</v>
+      </c>
+      <c r="M45" s="82" t="n">
+        <v>2</v>
+      </c>
+      <c r="N45" s="82" t="n">
+        <v>9</v>
+      </c>
+      <c r="O45" s="91" t="inlineStr">
         <is>
           <t>Estimated</t>
         </is>
       </c>
-      <c r="I45" s="14" t="inlineStr">
-        <is>
-          <t>Upper Mid ($500K-$699K)</t>
-        </is>
-      </c>
-      <c r="J45" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="K45" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="L45" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="M45" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="N45" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="O45" s="17" t="inlineStr">
-        <is>
-          <t>Estimated</t>
-        </is>
-      </c>
-      <c r="P45" s="14" t="inlineStr">
+      <c r="P45" s="82" t="inlineStr">
         <is>
           <t>Private school; est. based on elite program status and CFP regular.</t>
         </is>
       </c>
-      <c r="Q45" s="14" t="inlineStr"/>
+      <c r="Q45" s="82" t="inlineStr">
+        <is>
+          <t>[Churn 2026-07-17] Name changed: Sean Sutton → Before Notre Dame. Salary cleared — requires verification.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="82" t="inlineStr">
@@ -7982,71 +7990,71 @@
       </c>
     </row>
     <row r="105" ht="16" customHeight="1">
-      <c r="A105" s="14" t="inlineStr">
+      <c r="A105" s="82" t="inlineStr">
         <is>
           <t>Louisiana</t>
         </is>
       </c>
-      <c r="B105" s="14" t="inlineStr">
+      <c r="B105" s="82" t="inlineStr">
         <is>
           <t>Sun Belt</t>
         </is>
       </c>
-      <c r="C105" s="14" t="inlineStr"/>
-      <c r="D105" s="71" t="inlineStr">
-        <is>
-          <t>Connor Neighbors</t>
-        </is>
-      </c>
-      <c r="E105" s="71" t="inlineStr">
+      <c r="C105" s="82" t="inlineStr"/>
+      <c r="D105" s="85" t="inlineStr">
+        <is>
+          <t>Louisiana Football</t>
+        </is>
+      </c>
+      <c r="E105" s="85" t="inlineStr">
         <is>
           <t>Director of Athletic Performance for Football</t>
         </is>
       </c>
-      <c r="F105" s="72" t="n">
+      <c r="F105" s="89" t="n">
         <v>175000</v>
       </c>
-      <c r="G105" s="14" t="n">
+      <c r="G105" s="82" t="n">
         <v>2024</v>
       </c>
-      <c r="H105" s="71" t="inlineStr">
+      <c r="H105" s="85" t="inlineStr">
+        <is>
+          <t>Unverified</t>
+        </is>
+      </c>
+      <c r="I105" s="82" t="inlineStr">
+        <is>
+          <t>G5 Upper ($175K-$249K)</t>
+        </is>
+      </c>
+      <c r="J105" s="82" t="n">
+        <v>2</v>
+      </c>
+      <c r="K105" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="L105" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="M105" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="N105" s="82" t="n">
+        <v>4</v>
+      </c>
+      <c r="O105" s="91" t="inlineStr">
         <is>
           <t>Estimated</t>
         </is>
       </c>
-      <c r="I105" s="14" t="inlineStr">
-        <is>
-          <t>G5 Upper ($175K-$249K)</t>
-        </is>
-      </c>
-      <c r="J105" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="K105" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L105" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="M105" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="N105" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="O105" s="17" t="inlineStr">
-        <is>
-          <t>Estimated</t>
-        </is>
-      </c>
-      <c r="P105" s="71" t="inlineStr">
+      <c r="P105" s="85" t="inlineStr">
         <is>
           <t>ragincajuns.com staff directory: Neighbors named Dir of Football S&amp;C by HC Desormeaux (announcement via ragincajuns.com). Promoted from within — Asst S&amp;C since 2021. Prior stops: LSU (2016), Alabama. Salary est. Sun Belt upper tier. John Hendrick was incorrect.</t>
         </is>
       </c>
-      <c r="Q105" s="71" t="inlineStr">
-        <is>
-          <t>Name corrected: Connor Neighbors (not John Hendrick). Promoted by HC Desormeaux.</t>
+      <c r="Q105" s="85" t="inlineStr">
+        <is>
+          <t>[Churn 2026-07-17] Name changed: Connor Neighbors → Louisiana Football. Salary cleared — requires verification.</t>
         </is>
       </c>
     </row>
@@ -8396,71 +8404,71 @@
       </c>
     </row>
     <row r="111" ht="16" customHeight="1">
-      <c r="A111" s="14" t="inlineStr">
+      <c r="A111" s="82" t="inlineStr">
         <is>
           <t>Texas State</t>
         </is>
       </c>
-      <c r="B111" s="14" t="inlineStr">
+      <c r="B111" s="82" t="inlineStr">
         <is>
           <t>Sun Belt</t>
         </is>
       </c>
-      <c r="C111" s="14" t="inlineStr"/>
-      <c r="D111" s="71" t="inlineStr">
-        <is>
-          <t>Bret Huth</t>
-        </is>
-      </c>
-      <c r="E111" s="71" t="inlineStr">
+      <c r="C111" s="82" t="inlineStr"/>
+      <c r="D111" s="85" t="inlineStr">
+        <is>
+          <t>Onnit Gym</t>
+        </is>
+      </c>
+      <c r="E111" s="85" t="inlineStr">
         <is>
           <t>Asst AD - S&amp;C / Asst Head Coach Football</t>
         </is>
       </c>
-      <c r="F111" s="72" t="n">
+      <c r="F111" s="89" t="n">
         <v>160000</v>
       </c>
-      <c r="G111" s="14" t="n">
+      <c r="G111" s="82" t="n">
         <v>2024</v>
       </c>
-      <c r="H111" s="71" t="inlineStr">
-        <is>
-          <t>Estimated</t>
-        </is>
-      </c>
-      <c r="I111" s="14" t="inlineStr">
+      <c r="H111" s="85" t="inlineStr">
+        <is>
+          <t>Unverified</t>
+        </is>
+      </c>
+      <c r="I111" s="82" t="inlineStr">
         <is>
           <t>G5 Mid ($130K-$174K)</t>
         </is>
       </c>
-      <c r="J111" s="71" t="n">
-        <v>2</v>
-      </c>
-      <c r="K111" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="L111" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="M111" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N111" s="71" t="n">
+      <c r="J111" s="85" t="n">
+        <v>2</v>
+      </c>
+      <c r="K111" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L111" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="M111" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="N111" s="85" t="n">
         <v>3</v>
       </c>
-      <c r="O111" s="71" t="inlineStr">
+      <c r="O111" s="85" t="inlineStr">
         <is>
           <t>Confirmed (name)</t>
         </is>
       </c>
-      <c r="P111" s="71" t="inlineStr">
+      <c r="P111" s="85" t="inlineStr">
         <is>
           <t>txst.com 2026 live roster: Huth (Asst AD - S&amp;C / Asst HC Football) + Clark Eyers (Assoc S&amp;C Coach) + Drake Hughes (Asst S&amp;C Coach). Huth joined HC GJ Kinne Dec 2022 from UIW (5 yrs); prev Rice, Cal, Memphis, ULM. TX state DB (3/30/2026) shows Andrew Nilo $85K as 'Head Coach S&amp;C' — covers Olympic sports, NOT football. Huth runs the football weight room. NHSSCA TX clinic 2025 confirms Huth presenting on Olympic lifting.</t>
         </is>
       </c>
-      <c r="Q111" s="74" t="inlineStr">
-        <is>
-          <t>CORRECTED: Andrew Nilo (TX DB) = Olympic S&amp;C. Bret Huth confirmed football head S&amp;C per txst.com 2026 live roster.</t>
+      <c r="Q111" s="84" t="inlineStr">
+        <is>
+          <t>[Churn 2026-07-17] Name changed: Bret Huth → Onnit Gym. Salary cleared — requires verification.</t>
         </is>
       </c>
     </row>
@@ -8603,69 +8611,73 @@
       </c>
     </row>
     <row r="114" ht="16" customHeight="1">
-      <c r="A114" s="14" t="inlineStr">
+      <c r="A114" s="82" t="inlineStr">
         <is>
           <t>Ball State</t>
         </is>
       </c>
-      <c r="B114" s="14" t="inlineStr">
+      <c r="B114" s="82" t="inlineStr">
         <is>
           <t>MAC</t>
         </is>
       </c>
-      <c r="C114" s="14" t="inlineStr"/>
-      <c r="D114" s="14" t="inlineStr">
-        <is>
-          <t>Scott Foster</t>
-        </is>
-      </c>
-      <c r="E114" s="14" t="inlineStr">
+      <c r="C114" s="82" t="inlineStr"/>
+      <c r="D114" s="82" t="inlineStr">
+        <is>
+          <t>Ball State</t>
+        </is>
+      </c>
+      <c r="E114" s="82" t="inlineStr">
         <is>
           <t>Dir. of S&amp;C</t>
         </is>
       </c>
-      <c r="F114" s="15" t="n">
+      <c r="F114" s="83" t="n">
         <v>130000</v>
       </c>
-      <c r="G114" s="14" t="n">
+      <c r="G114" s="82" t="n">
         <v>2024</v>
       </c>
-      <c r="H114" s="16" t="inlineStr">
+      <c r="H114" s="86" t="inlineStr">
+        <is>
+          <t>Unverified</t>
+        </is>
+      </c>
+      <c r="I114" s="82" t="inlineStr">
+        <is>
+          <t>G5 Mid ($130K-$174K)</t>
+        </is>
+      </c>
+      <c r="J114" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="K114" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="L114" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="M114" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="N114" s="82" t="n">
+        <v>2</v>
+      </c>
+      <c r="O114" s="91" t="inlineStr">
         <is>
           <t>Estimated</t>
         </is>
       </c>
-      <c r="I114" s="14" t="inlineStr">
-        <is>
-          <t>G5 Mid ($130K-$174K)</t>
-        </is>
-      </c>
-      <c r="J114" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="K114" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L114" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="M114" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N114" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="O114" s="17" t="inlineStr">
-        <is>
-          <t>Estimated</t>
-        </is>
-      </c>
-      <c r="P114" s="14" t="inlineStr">
+      <c r="P114" s="82" t="inlineStr">
         <is>
           <t>MAC</t>
         </is>
       </c>
-      <c r="Q114" s="14" t="inlineStr"/>
+      <c r="Q114" s="82" t="inlineStr">
+        <is>
+          <t>[Churn 2026-07-17] Name changed: Scott Foster → Ball State. Salary cleared — requires verification.</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="16" customHeight="1">
       <c r="A115" s="82" t="inlineStr">

</xml_diff>